<commit_message>
TF -> TD: the acronym now matches the words
TF was chosen to preserve the F from "Design Foundation", but Foundation was
inherited vagueness. The document defines the tool, so Tool Definition is what it
is - and TD is the honest initialism. TD.1 pairs with TSP.1 as cleanly as TF.1 did.

Done now rather than later: nothing is adopted yet, so the cost is four file
renames and their references. After adoption it would be a breaking change to
every cross-reference.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/registry/TSP Register.xlsx
+++ b/registry/TSP Register.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>TSP/TSP.1 WBS Register/TF.1 - WBS Register.md</t>
+          <t>TSP/TSP.1 WBS Register/TD.1 - WBS Register.md</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>TSP/TSP.2 RAID Register/TF.2 - RAID Register.md</t>
+          <t>TSP/TSP.2 RAID Register/TD.2 - RAID Register.md</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>TSP/TSP.3 TSP Register/TF.3 - TSP Register.md</t>
+          <t>TSP/TSP.3 TSP Register/TD.3 - TSP Register.md</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">

</xml_diff>